<commit_message>
Actualizar datos 2026 (2026-04-20 PM)
</commit_message>
<xml_diff>
--- a/data/asistencia/Dorados 2026.xlsx
+++ b/data/asistencia/Dorados 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>80.07%</t>
+    <t>89.83%</t>
   </si>
   <si>
     <t>Jardin Izquierdo</t>
   </si>
   <si>
-    <t>50.86%</t>
+    <t>57.19%</t>
   </si>
   <si>
     <t>Oro</t>
@@ -109,13 +109,10 @@
     <t>Plata</t>
   </si>
   <si>
-    <t>99.94%</t>
-  </si>
-  <si>
     <t>Preferente</t>
   </si>
   <si>
-    <t>98.87%</t>
+    <t>98.97%</t>
   </si>
   <si>
     <t>Suite Premier</t>
@@ -133,7 +130,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>80.10%</t>
+    <t>83.26%</t>
   </si>
 </sst>
 </file>
@@ -646,13 +643,13 @@
         <v>1515</v>
       </c>
       <c r="C6" s="6">
-        <v>909</v>
+        <v>1044</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="6">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
@@ -685,10 +682,10 @@
         <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>1213</v>
+        <v>1361</v>
       </c>
       <c r="Q6" s="6">
-        <v>302</v>
+        <v>154</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -702,13 +699,13 @@
         <v>1516</v>
       </c>
       <c r="C7" s="6">
-        <v>458</v>
+        <v>554</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="6">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>22</v>
@@ -735,16 +732,16 @@
         <v>22</v>
       </c>
       <c r="N7" s="6">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="O7" s="6">
         <v>2</v>
       </c>
       <c r="P7" s="6">
-        <v>771</v>
+        <v>867</v>
       </c>
       <c r="Q7" s="6">
-        <v>745</v>
+        <v>649</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -926,13 +923,13 @@
         <v>1709</v>
       </c>
       <c r="C11" s="6">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="6">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
@@ -959,36 +956,36 @@
         <v>22</v>
       </c>
       <c r="N11" s="6">
-        <v>653</v>
+        <v>644</v>
       </c>
       <c r="O11" s="6">
         <v>4</v>
       </c>
       <c r="P11" s="6">
-        <v>1708</v>
-      </c>
-      <c r="Q11" s="6">
-        <v>1</v>
+        <v>1709</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="6">
         <v>1853</v>
       </c>
       <c r="C12" s="6">
-        <v>1577</v>
+        <v>1579</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
@@ -1015,24 +1012,24 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>1832</v>
+        <v>1834</v>
       </c>
       <c r="Q12" s="6">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="6">
         <v>128</v>
@@ -1055,8 +1052,8 @@
       <c r="H13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="6" t="s">
-        <v>22</v>
+      <c r="I13" s="6">
+        <v>15</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>22</v>
@@ -1073,8 +1070,8 @@
       <c r="N13" s="6">
         <v>36</v>
       </c>
-      <c r="O13" s="6">
-        <v>15</v>
+      <c r="O13" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P13" s="6">
         <v>51</v>
@@ -1083,12 +1080,12 @@
         <v>77</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="6">
         <v>400</v>
@@ -1139,12 +1136,12 @@
         <v>400</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15" s="7">
         <f>SUM(B6:B14)</f>
@@ -1195,7 +1192,7 @@
         <f>SUM(Q6:Q14)</f>
       </c>
       <c r="R15" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update 2026 data from local files (Boletomóvil reports Apr 21)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/asistencia/Dorados 2026.xlsx
+++ b/data/asistencia/Dorados 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>89.83%</t>
+    <t>95.51%</t>
   </si>
   <si>
     <t>Jardin Izquierdo</t>
   </si>
   <si>
-    <t>57.19%</t>
+    <t>64.38%</t>
   </si>
   <si>
     <t>Oro</t>
@@ -112,7 +112,7 @@
     <t>Preferente</t>
   </si>
   <si>
-    <t>98.97%</t>
+    <t>99.46%</t>
   </si>
   <si>
     <t>Suite Premier</t>
@@ -130,7 +130,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>83.26%</t>
+    <t>85.87%</t>
   </si>
 </sst>
 </file>
@@ -643,7 +643,7 @@
         <v>1515</v>
       </c>
       <c r="C6" s="6">
-        <v>1044</v>
+        <v>1123</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
@@ -678,14 +678,14 @@
       <c r="N6" s="6">
         <v>188</v>
       </c>
-      <c r="O6" s="6" t="s">
-        <v>22</v>
+      <c r="O6" s="6">
+        <v>7</v>
       </c>
       <c r="P6" s="6">
-        <v>1361</v>
+        <v>1447</v>
       </c>
       <c r="Q6" s="6">
-        <v>154</v>
+        <v>68</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +699,7 @@
         <v>1516</v>
       </c>
       <c r="C7" s="6">
-        <v>554</v>
+        <v>662</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -735,13 +735,13 @@
         <v>176</v>
       </c>
       <c r="O7" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6">
-        <v>867</v>
+        <v>976</v>
       </c>
       <c r="Q7" s="6">
-        <v>649</v>
+        <v>540</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -929,7 +929,7 @@
         <v>22</v>
       </c>
       <c r="E11" s="6">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
@@ -941,7 +941,7 @@
         <v>22</v>
       </c>
       <c r="I11" s="6">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>22</v>
@@ -979,7 +979,7 @@
         <v>1853</v>
       </c>
       <c r="C12" s="6">
-        <v>1579</v>
+        <v>1588</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
@@ -1018,10 +1018,10 @@
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>1834</v>
+        <v>1843</v>
       </c>
       <c r="Q12" s="6">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Update 2026 data (Apr 22)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/asistencia/Dorados 2026.xlsx
+++ b/data/asistencia/Dorados 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="39">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,13 +82,13 @@
     <t>-</t>
   </si>
   <si>
-    <t>95.51%</t>
+    <t>98.09%</t>
   </si>
   <si>
     <t>Jardin Izquierdo</t>
   </si>
   <si>
-    <t>64.38%</t>
+    <t>77.97%</t>
   </si>
   <si>
     <t>Oro</t>
@@ -112,9 +112,6 @@
     <t>Preferente</t>
   </si>
   <si>
-    <t>99.46%</t>
-  </si>
-  <si>
     <t>Suite Premier</t>
   </si>
   <si>
@@ -130,7 +127,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>85.87%</t>
+    <t>89.13%</t>
   </si>
 </sst>
 </file>
@@ -643,13 +640,13 @@
         <v>1515</v>
       </c>
       <c r="C6" s="6">
-        <v>1123</v>
+        <v>1167</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="6">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
@@ -676,16 +673,16 @@
         <v>22</v>
       </c>
       <c r="N6" s="6">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="O6" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P6" s="6">
-        <v>1447</v>
+        <v>1486</v>
       </c>
       <c r="Q6" s="6">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -699,7 +696,7 @@
         <v>1516</v>
       </c>
       <c r="C7" s="6">
-        <v>662</v>
+        <v>870</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
@@ -735,13 +732,13 @@
         <v>176</v>
       </c>
       <c r="O7" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P7" s="6">
-        <v>976</v>
+        <v>1182</v>
       </c>
       <c r="Q7" s="6">
-        <v>540</v>
+        <v>334</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -760,8 +757,8 @@
       <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>22</v>
+      <c r="E8" s="6">
+        <v>20</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>22</v>
@@ -788,7 +785,7 @@
         <v>22</v>
       </c>
       <c r="N8" s="6">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="O8" s="6" t="s">
         <v>22</v>
@@ -885,7 +882,7 @@
         <v>22</v>
       </c>
       <c r="I10" s="6">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>22</v>
@@ -900,7 +897,7 @@
         <v>22</v>
       </c>
       <c r="N10" s="6">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="O10" s="6" t="s">
         <v>22</v>
@@ -923,13 +920,13 @@
         <v>1709</v>
       </c>
       <c r="C11" s="6">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="6">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
@@ -941,7 +938,7 @@
         <v>22</v>
       </c>
       <c r="I11" s="6">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>22</v>
@@ -956,10 +953,10 @@
         <v>22</v>
       </c>
       <c r="N11" s="6">
-        <v>644</v>
+        <v>598</v>
       </c>
       <c r="O11" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P11" s="6">
         <v>1709</v>
@@ -979,13 +976,13 @@
         <v>1853</v>
       </c>
       <c r="C12" s="6">
-        <v>1588</v>
+        <v>1597</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
@@ -1012,24 +1009,24 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>127</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>22</v>
+        <v>120</v>
+      </c>
+      <c r="O12" s="6">
+        <v>1</v>
       </c>
       <c r="P12" s="6">
-        <v>1843</v>
-      </c>
-      <c r="Q12" s="6">
-        <v>10</v>
+        <v>1853</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="6">
         <v>128</v>
@@ -1080,12 +1077,12 @@
         <v>77</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="6">
         <v>400</v>
@@ -1136,12 +1133,12 @@
         <v>400</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" s="7">
         <f>SUM(B6:B14)</f>
@@ -1192,7 +1189,7 @@
         <f>SUM(Q6:Q14)</f>
       </c>
       <c r="R15" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update 2026 data (Apr 23)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/asistencia/Dorados 2026.xlsx
+++ b/data/asistencia/Dorados 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="41">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -76,19 +76,25 @@
     <t>% OCUPACIÓN</t>
   </si>
   <si>
+    <t>Grada Sol</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>0.82%</t>
+  </si>
+  <si>
     <t>Jardin Derecho</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>98.09%</t>
+    <t>99.27%</t>
   </si>
   <si>
     <t>Jardin Izquierdo</t>
   </si>
   <si>
-    <t>77.97%</t>
+    <t>95.84%</t>
   </si>
   <si>
     <t>Oro</t>
@@ -127,7 +133,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>89.13%</t>
+    <t>54.83%</t>
   </si>
 </sst>
 </file>
@@ -549,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -637,16 +643,16 @@
         <v>21</v>
       </c>
       <c r="B6" s="6">
-        <v>1515</v>
+        <v>5500</v>
       </c>
       <c r="C6" s="6">
-        <v>1167</v>
+        <v>45</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="6">
-        <v>139</v>
+      <c r="E6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
@@ -672,17 +678,17 @@
       <c r="M6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="N6" s="6">
-        <v>178</v>
-      </c>
-      <c r="O6" s="6">
-        <v>2</v>
+      <c r="N6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P6" s="6">
-        <v>1486</v>
+        <v>45</v>
       </c>
       <c r="Q6" s="6">
-        <v>29</v>
+        <v>5455</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -693,16 +699,16 @@
         <v>24</v>
       </c>
       <c r="B7" s="6">
-        <v>1516</v>
+        <v>1515</v>
       </c>
       <c r="C7" s="6">
-        <v>870</v>
+        <v>1187</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="6">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>22</v>
@@ -729,16 +735,16 @@
         <v>22</v>
       </c>
       <c r="N7" s="6">
-        <v>176</v>
-      </c>
-      <c r="O7" s="6">
-        <v>1</v>
+        <v>143</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P7" s="6">
-        <v>1182</v>
+        <v>1504</v>
       </c>
       <c r="Q7" s="6">
-        <v>334</v>
+        <v>11</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -749,28 +755,28 @@
         <v>26</v>
       </c>
       <c r="B8" s="6">
-        <v>174</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>22</v>
+        <v>1516</v>
+      </c>
+      <c r="C8" s="6">
+        <v>1141</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="6">
-        <v>20</v>
+        <v>145</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="6">
-        <v>12</v>
+      <c r="G8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="6">
-        <v>60</v>
+      <c r="I8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>22</v>
@@ -785,16 +791,16 @@
         <v>22</v>
       </c>
       <c r="N8" s="6">
-        <v>82</v>
-      </c>
-      <c r="O8" s="6" t="s">
-        <v>22</v>
+        <v>166</v>
+      </c>
+      <c r="O8" s="6">
+        <v>1</v>
       </c>
       <c r="P8" s="6">
-        <v>174</v>
-      </c>
-      <c r="Q8" s="6" t="s">
-        <v>22</v>
+        <v>1453</v>
+      </c>
+      <c r="Q8" s="6">
+        <v>63</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>27</v>
@@ -805,7 +811,7 @@
         <v>28</v>
       </c>
       <c r="B9" s="6">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>22</v>
@@ -813,103 +819,103 @@
       <c r="D9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>22</v>
+      <c r="E9" s="6">
+        <v>20</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="6">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I9" s="6">
+        <v>60</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N9" s="6">
         <v>82</v>
       </c>
-      <c r="J9" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N9" s="6">
-        <v>40</v>
-      </c>
       <c r="O9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P9" s="6">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="Q9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="6">
+        <v>164</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="6">
+        <v>42</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="6">
+        <v>82</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N10" s="6">
+        <v>40</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P10" s="6">
+        <v>164</v>
+      </c>
+      <c r="Q10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="R10" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="B10" s="6">
-        <v>360</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="6">
-        <v>41</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="6">
-        <v>199</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N10" s="6">
-        <v>110</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="P10" s="6">
-        <v>350</v>
-      </c>
-      <c r="Q10" s="6">
-        <v>10</v>
-      </c>
-      <c r="R10" s="6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -917,28 +923,28 @@
         <v>31</v>
       </c>
       <c r="B11" s="6">
-        <v>1709</v>
-      </c>
-      <c r="C11" s="6">
-        <v>839</v>
+        <v>360</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="6">
-        <v>162</v>
+      <c r="E11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G11" s="6">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="6">
-        <v>52</v>
+        <v>199</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>22</v>
@@ -953,48 +959,48 @@
         <v>22</v>
       </c>
       <c r="N11" s="6">
-        <v>598</v>
-      </c>
-      <c r="O11" s="6">
-        <v>3</v>
+        <v>110</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P11" s="6">
-        <v>1709</v>
-      </c>
-      <c r="Q11" s="6" t="s">
-        <v>22</v>
+        <v>350</v>
+      </c>
+      <c r="Q11" s="6">
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="6">
-        <v>1853</v>
+        <v>1709</v>
       </c>
       <c r="C12" s="6">
-        <v>1597</v>
+        <v>842</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>130</v>
+        <v>186</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="6">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>22</v>
+      <c r="I12" s="6">
+        <v>52</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>22</v>
@@ -1009,48 +1015,48 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>120</v>
-      </c>
-      <c r="O12" s="6">
-        <v>1</v>
+        <v>574</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>1853</v>
+        <v>1709</v>
       </c>
       <c r="Q12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="6">
-        <v>128</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>22</v>
+        <v>1853</v>
+      </c>
+      <c r="C13" s="6">
+        <v>1598</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>22</v>
+      <c r="E13" s="6">
+        <v>130</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="6" t="s">
-        <v>22</v>
+      <c r="G13" s="6">
+        <v>5</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="6">
-        <v>15</v>
+      <c r="I13" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>22</v>
@@ -1065,19 +1071,19 @@
         <v>22</v>
       </c>
       <c r="N13" s="6">
-        <v>36</v>
+        <v>120</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>51</v>
-      </c>
-      <c r="Q13" s="6">
-        <v>77</v>
+        <v>1853</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1085,7 +1091,7 @@
         <v>35</v>
       </c>
       <c r="B14" s="6">
-        <v>400</v>
+        <v>128</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>22</v>
@@ -1105,8 +1111,8 @@
       <c r="H14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>22</v>
+      <c r="I14" s="6">
+        <v>15</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>22</v>
@@ -1120,80 +1126,136 @@
       <c r="M14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="N14" s="6" t="s">
-        <v>22</v>
+      <c r="N14" s="6">
+        <v>36</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="6" t="s">
-        <v>22</v>
+      <c r="P14" s="6">
+        <v>51</v>
       </c>
       <c r="Q14" s="6">
-        <v>400</v>
+        <v>77</v>
       </c>
       <c r="R14" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="7">
-        <f>SUM(B6:B14)</f>
-      </c>
-      <c r="C15" s="7">
-        <f>SUM(C6:C14)</f>
-      </c>
-      <c r="D15" s="7">
-        <f>SUM(D6:D14)</f>
-      </c>
-      <c r="E15" s="7">
-        <f>SUM(E6:E14)</f>
-      </c>
-      <c r="F15" s="7">
-        <f>SUM(F6:F14)</f>
-      </c>
-      <c r="G15" s="7">
-        <f>SUM(G6:G14)</f>
-      </c>
-      <c r="H15" s="7">
-        <f>SUM(H6:H14)</f>
-      </c>
-      <c r="I15" s="7">
-        <f>SUM(I6:I14)</f>
-      </c>
-      <c r="J15" s="7">
-        <f>SUM(J6:J14)</f>
-      </c>
-      <c r="K15" s="7">
-        <f>SUM(K6:K14)</f>
-      </c>
-      <c r="L15" s="7">
-        <f>SUM(L6:L14)</f>
-      </c>
-      <c r="M15" s="7">
-        <f>SUM(M6:M14)</f>
-      </c>
-      <c r="N15" s="7">
-        <f>SUM(N6:N14)</f>
-      </c>
-      <c r="O15" s="7">
-        <f>SUM(O6:O14)</f>
-      </c>
-      <c r="P15" s="7">
-        <f>SUM(P6:P14)</f>
-      </c>
-      <c r="Q15" s="7">
-        <f>SUM(Q6:Q14)</f>
-      </c>
-      <c r="R15" s="7" t="s">
+      <c r="B15" s="6">
+        <v>400</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q15" s="6">
+        <v>400</v>
+      </c>
+      <c r="R15" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="7">
+        <f>SUM(B6:B15)</f>
+      </c>
+      <c r="C16" s="7">
+        <f>SUM(C6:C15)</f>
+      </c>
+      <c r="D16" s="7">
+        <f>SUM(D6:D15)</f>
+      </c>
+      <c r="E16" s="7">
+        <f>SUM(E6:E15)</f>
+      </c>
+      <c r="F16" s="7">
+        <f>SUM(F6:F15)</f>
+      </c>
+      <c r="G16" s="7">
+        <f>SUM(G6:G15)</f>
+      </c>
+      <c r="H16" s="7">
+        <f>SUM(H6:H15)</f>
+      </c>
+      <c r="I16" s="7">
+        <f>SUM(I6:I15)</f>
+      </c>
+      <c r="J16" s="7">
+        <f>SUM(J6:J15)</f>
+      </c>
+      <c r="K16" s="7">
+        <f>SUM(K6:K15)</f>
+      </c>
+      <c r="L16" s="7">
+        <f>SUM(L6:L15)</f>
+      </c>
+      <c r="M16" s="7">
+        <f>SUM(M6:M15)</f>
+      </c>
+      <c r="N16" s="7">
+        <f>SUM(N6:N15)</f>
+      </c>
+      <c r="O16" s="7">
+        <f>SUM(O6:O15)</f>
+      </c>
+      <c r="P16" s="7">
+        <f>SUM(P6:P15)</f>
+      </c>
+      <c r="Q16" s="7">
+        <f>SUM(Q6:Q15)</f>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026 data (Apr 24)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/asistencia/Dorados 2026.xlsx
+++ b/data/asistencia/Dorados 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -82,27 +82,21 @@
     <t>-</t>
   </si>
   <si>
-    <t>0.82%</t>
+    <t>8.22%</t>
   </si>
   <si>
     <t>Jardin Derecho</t>
   </si>
   <si>
-    <t>99.27%</t>
+    <t>100.00%</t>
   </si>
   <si>
     <t>Jardin Izquierdo</t>
   </si>
   <si>
-    <t>95.84%</t>
-  </si>
-  <si>
     <t>Oro</t>
   </si>
   <si>
-    <t>100.00%</t>
-  </si>
-  <si>
     <t>Palcos Dorados</t>
   </si>
   <si>
@@ -133,7 +127,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>54.83%</t>
+    <t>58.44%</t>
   </si>
 </sst>
 </file>
@@ -646,13 +640,13 @@
         <v>5500</v>
       </c>
       <c r="C6" s="6">
-        <v>45</v>
+        <v>440</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>22</v>
+      <c r="E6" s="6">
+        <v>8</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
@@ -681,14 +675,14 @@
       <c r="N6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="O6" s="6" t="s">
-        <v>22</v>
+      <c r="O6" s="6">
+        <v>4</v>
       </c>
       <c r="P6" s="6">
-        <v>45</v>
+        <v>452</v>
       </c>
       <c r="Q6" s="6">
-        <v>5455</v>
+        <v>5048</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>23</v>
@@ -702,13 +696,13 @@
         <v>1515</v>
       </c>
       <c r="C7" s="6">
-        <v>1187</v>
+        <v>1198</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="6">
-        <v>174</v>
+        <v>244</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>22</v>
@@ -735,16 +729,16 @@
         <v>22</v>
       </c>
       <c r="N7" s="6">
-        <v>143</v>
+        <v>73</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P7" s="6">
-        <v>1504</v>
-      </c>
-      <c r="Q7" s="6">
-        <v>11</v>
+        <v>1515</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -758,13 +752,13 @@
         <v>1516</v>
       </c>
       <c r="C8" s="6">
-        <v>1141</v>
+        <v>1205</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="6">
-        <v>145</v>
+        <v>254</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>22</v>
@@ -791,24 +785,24 @@
         <v>22</v>
       </c>
       <c r="N8" s="6">
-        <v>166</v>
-      </c>
-      <c r="O8" s="6">
-        <v>1</v>
+        <v>57</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="P8" s="6">
-        <v>1453</v>
-      </c>
-      <c r="Q8" s="6">
-        <v>63</v>
+        <v>1516</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="6">
         <v>174</v>
@@ -820,7 +814,7 @@
         <v>22</v>
       </c>
       <c r="E9" s="6">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>22</v>
@@ -832,7 +826,7 @@
         <v>22</v>
       </c>
       <c r="I9" s="6">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>22</v>
@@ -847,7 +841,7 @@
         <v>22</v>
       </c>
       <c r="N9" s="6">
-        <v>82</v>
+        <v>30</v>
       </c>
       <c r="O9" s="6" t="s">
         <v>22</v>
@@ -859,12 +853,12 @@
         <v>22</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B10" s="6">
         <v>164</v>
@@ -915,12 +909,12 @@
         <v>22</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B11" s="6">
         <v>360</v>
@@ -971,36 +965,36 @@
         <v>10</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B12" s="6">
         <v>1709</v>
       </c>
       <c r="C12" s="6">
-        <v>842</v>
+        <v>861</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="6">
-        <v>186</v>
+        <v>228</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="6">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="I12" s="6">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>22</v>
@@ -1015,7 +1009,7 @@
         <v>22</v>
       </c>
       <c r="N12" s="6">
-        <v>574</v>
+        <v>512</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>22</v>
@@ -1027,12 +1021,12 @@
         <v>22</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B13" s="6">
         <v>1853</v>
@@ -1083,12 +1077,12 @@
         <v>22</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B14" s="6">
         <v>128</v>
@@ -1139,12 +1133,12 @@
         <v>77</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B15" s="6">
         <v>400</v>
@@ -1195,12 +1189,12 @@
         <v>400</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" s="7">
         <f>SUM(B6:B15)</f>
@@ -1251,7 +1245,7 @@
         <f>SUM(Q6:Q15)</f>
       </c>
       <c r="R16" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>